<commit_message>
Add reliance-posture hedge (CB-10): terms page, CONTRACT clause, export-side notice
Measured baseline: 104/155 tools citing regulation carried no hedge, only 12
had a disclaimer div, no estate-wide terms page existed, CONTRACT.md said
"advice" zero times.

- disclosures/terms.html: estate-wide reliance/terms page, linked from
  disclosures/index.html and the shared root/node footer (_page-chrome.mjs).
- CONTRACT.md Amendment A9: additive clause requiring a reliance hedge on any
  surface citing regulation, and requiring exports to carry it.
- chaingraph/exporters/_meta.mjs: reliance_notice added to metaBlock() so
  every §13 export profile embeds it (csv/xlsx/pdf/vc/xbrl/index metadata);
  explicit visible line added to pdf.mjs and xlsx.mjs.

104-tool retrofit is out of scope (separate future work unit, not silently
dropped). No coverage-ratio gate added, per CLAUSE-BINDING-BUILD-SPEC.md §12.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/chaingraph/exporters/sample-export.xlsx
+++ b/chaingraph/exporters/sample-export.xlsx
@@ -147,6 +147,14 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not legal, investment, tax, or compliance advice. A computed view of the cited authority as of generated_at, not a substitute for review by a qualified advisor against the current official source text.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add reliance-posture hedge (CB-10): terms page, CONTRACT clause, export-side notice (#921)
Measured baseline: 104/155 tools citing regulation carried no hedge, only 12
had a disclaimer div, no estate-wide terms page existed, CONTRACT.md said
"advice" zero times.

- disclosures/terms.html: estate-wide reliance/terms page, linked from
  disclosures/index.html and the shared root/node footer (_page-chrome.mjs).
- CONTRACT.md Amendment A9: additive clause requiring a reliance hedge on any
  surface citing regulation, and requiring exports to carry it.
- chaingraph/exporters/_meta.mjs: reliance_notice added to metaBlock() so
  every §13 export profile embeds it (csv/xlsx/pdf/vc/xbrl/index metadata);
  explicit visible line added to pdf.mjs and xlsx.mjs.

104-tool retrofit is out of scope (separate future work unit, not silently
dropped). No coverage-ratio gate added, per CLAUSE-BINDING-BUILD-SPEC.md §12.

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/chaingraph/exporters/sample-export.xlsx
+++ b/chaingraph/exporters/sample-export.xlsx
@@ -147,6 +147,14 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not legal, investment, tax, or compliance advice. A computed view of the cited authority as of generated_at, not a substitute for review by a qualified advisor against the current official source text.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>

</xml_diff>